<commit_message>
made pi even flatter, updated bom
</commit_message>
<xml_diff>
--- a/Other/Current BOM.xlsx
+++ b/Other/Current BOM.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\grtis\Documents\PiHome\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\grtis\Documents\PiHome\Other\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFBD1852-3E3E-4D7F-A580-33709C28E9FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D73CCEB-7B65-43C6-B839-C1A8A64C9665}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21840" xr2:uid="{45E5082E-FD5C-4A39-94F7-261BF944CA5F}"/>
   </bookViews>
@@ -68,13 +68,13 @@
     <t>Monitor</t>
   </si>
   <si>
-    <t>Right Angle Mini HDMI</t>
-  </si>
-  <si>
-    <t>USD</t>
-  </si>
-  <si>
-    <t>n</t>
+    <t>Cable</t>
+  </si>
+  <si>
+    <t>Mini HDMI C4</t>
+  </si>
+  <si>
+    <t>Micro HDMI D3</t>
   </si>
 </sst>
 </file>
@@ -141,16 +141,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="7" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="7" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill>
@@ -165,13 +165,6 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -183,6 +176,149 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>376671</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>92913</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{356D38E7-6CA6-1EAA-B8BF-DA5DA0B19C8E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3822989" y="190501"/>
+          <a:ext cx="4039466" cy="2378912"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>42957</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>171120</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>473877</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>125640</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="5" name="Ink 4">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0B432B35-AC2E-2125-51A4-E7E01D2986AF}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="3255480" y="933120"/>
+            <a:ext cx="430920" cy="335520"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="5" name="Ink 4">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0B432B35-AC2E-2125-51A4-E7E01D2986AF}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="3249360" y="927000"/>
+              <a:ext cx="443160" cy="347760"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/ink/ink1.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-06-05T05:31:37.022"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#E71224"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 451 24575,'57'-3'0,"80"-13"0,-114 13 0,19-5 0,83-28 0,-119 34 0,59-21 0,-1-2 0,-1-4 0,87-53 0,63-33 0,-172 92 0,1 1 0,1 2 0,46-14 0,-61 27-1365,-20 4-5461</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="936.88">121 932 24575,'7'-1'0,"0"-1"0,-1 1 0,1-1 0,-1 0 0,0-1 0,10-4 0,18-7 0,71-18 0,151-69 0,-175 67 0,139-40 0,68-22 0,-272 88-1365,-9 4-5461</inkml:trace>
+</inkml:ink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -502,7 +638,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{944B7241-5C83-4031-8AB1-AE0A1A86B581}">
-  <dimension ref="B2:G6"/>
+  <dimension ref="B2:G7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
@@ -512,12 +648,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
     </row>
     <row r="3" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
@@ -558,16 +694,15 @@
       </c>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="C6" s="3">
-        <v>6.5</v>
       </c>
       <c r="D6" t="s">
         <v>10</v>
       </c>
-      <c r="E6" t="s">
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D7" t="s">
         <v>11</v>
       </c>
     </row>
@@ -576,16 +711,14 @@
     <mergeCell ref="B2:E2"/>
   </mergeCells>
   <conditionalFormatting sqref="B1:E1048576">
-    <cfRule type="expression" dxfId="2" priority="2">
-      <formula>$E1="y"</formula>
-    </cfRule>
     <cfRule type="expression" dxfId="1" priority="1">
       <formula>$E1="n"</formula>
     </cfRule>
+    <cfRule type="expression" dxfId="0" priority="2">
+      <formula>$E1="y"</formula>
+    </cfRule>
   </conditionalFormatting>
-  <hyperlinks>
-    <hyperlink ref="B6" r:id="rId1" xr:uid="{EBC32FCC-EF46-4CEC-8257-7477B4BC216B}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>